<commit_message>
docs: add PRD, BRD, RFP, and process-diagram PDFs for Zia
Zia accepts standard requirement attachments. Add Product, Business, and
RFP PDFs plus six process diagrams so the Creator recon app can be built
from those slots, with Excel fallback.

Co-authored-by: googrlc <googrlc@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/docs/zoho-creator/ZIA_UPLOAD.xlsx
+++ b/docs/zoho-creator/ZIA_UPLOAD.xlsx
@@ -469,10 +469,13 @@
           <t xml:space="preserve"># Zia prompt — paste this first
 You are building a Zoho Creator application for Risk Solutions Group (RSG)
 called **RSG Policy Reconciliation**.
-Zia file upload accepts only: .xls .xlsx .xlsm .csv .tsv .ods .mdb .accdb
-.ds .json .numbers (max 2 GB; over 100 MB must be CSV). Do **not** wait for
-Markdown. Upload **one** file: `ZIA_UPLOAD.xlsx` (or `ZIA_UPLOAD.json` /
-`ZIA_UPLOAD.csv`). That file is the full specification.
+Zia can attach PRD, BRD, RFP, and process diagrams. Attach these four PDFs:
+- `PRD_RSG_Policy_Reconciliation.pdf`
+- `BRD_RSG_Policy_Reconciliation.pdf`
+- `RFP_RSG_Policy_Reconciliation.pdf`
+- `PROCESS_DIAGRAMS_RSG_Policy_Reconciliation.pdf`
+Also upload `ZIA_UPLOAD.xlsx` as the field dictionary and Deluge appendix.
+Do not invent fields or verdicts. Build **Phase 1 only**, then stop.
 Read those uploads as the only source of truth (`zia_prompt`,
 `specification_markdown`, `forms`, `picklists`, `deluge`, `sample_records`).
 Build the application **exactly** as specified.

</xml_diff>

<commit_message>
docs: combine Zia requirements into one ZIA_UPLOAD.pdf
Zia allows a single attachment. Merge PRD, BRD, RFP, process diagrams,
field dictionaries, picklists, Deluge, and seed cases into ZIA_UPLOAD.pdf.

Co-authored-by: googrlc <googrlc@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/docs/zoho-creator/ZIA_UPLOAD.xlsx
+++ b/docs/zoho-creator/ZIA_UPLOAD.xlsx
@@ -469,13 +469,9 @@
           <t xml:space="preserve"># Zia prompt — paste this first
 You are building a Zoho Creator application for Risk Solutions Group (RSG)
 called **RSG Policy Reconciliation**.
-Zia can attach PRD, BRD, RFP, and process diagrams. Attach these four PDFs:
-- `PRD_RSG_Policy_Reconciliation.pdf`
-- `BRD_RSG_Policy_Reconciliation.pdf`
-- `RFP_RSG_Policy_Reconciliation.pdf`
-- `PROCESS_DIAGRAMS_RSG_Policy_Reconciliation.pdf`
-Also upload `ZIA_UPLOAD.xlsx` as the field dictionary and Deluge appendix.
-Do not invent fields or verdicts. Build **Phase 1 only**, then stop.
+You are attaching **one document**: `ZIA_UPLOAD.pdf`. It is the complete
+package (PRD + BRD + RFP + process diagrams + field dictionaries + Deluge).
+Build Phase 1 only, then stop.
 Read those uploads as the only source of truth (`zia_prompt`,
 `specification_markdown`, `forms`, `picklists`, `deluge`, `sample_records`).
 Build the application **exactly** as specified.

</xml_diff>